<commit_message>
T-1546: probe lifted INDEX over a cached external range; file T-1554
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gyNXdXoDF2bstugfMeBDr
</commit_message>
<xml_diff>
--- a/eval/suites/fixtures/cases/external-link-cached-ranges.xlsx
+++ b/eval/suites/fixtures/cases/external-link-cached-ranges.xlsx
@@ -1334,6 +1334,137 @@
         <v>0</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>IDXlift11</t>
+        </is>
+      </c>
+      <c r="B83">
+        <f t="array" ref="B83:C83">INDEX([1]Uses!$A$1:$B$3,{1,2},1)</f>
+        <v>0</v>
+      </c>
+      <c r="C83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>IDXlift22</t>
+        </is>
+      </c>
+      <c r="B84">
+        <f t="array" ref="B84:C84">INDEX([1]Uses!$A$1:$B$3,{2,3},2)</f>
+        <v>0</v>
+      </c>
+      <c r="C84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>IDXliftWholeCol</t>
+        </is>
+      </c>
+      <c r="B85">
+        <f t="array" ref="B85:C85">INDEX([1]Uses!$A$1:$B$3,{0,2},1)</f>
+        <v>0</v>
+      </c>
+      <c r="C85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>IDXliftWholeRow</t>
+        </is>
+      </c>
+      <c r="B86">
+        <f t="array" ref="B86:C86">INDEX([1]Uses!$A$1:$B$3,{1,2},0)</f>
+        <v>0</v>
+      </c>
+      <c r="C86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>IDXliftOOR</t>
+        </is>
+      </c>
+      <c r="B87">
+        <f t="array" ref="B87:C87">INDEX([1]Uses!$A$1:$B$3,{1,4},1)</f>
+        <v>0</v>
+      </c>
+      <c r="C87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>IDXliftErrCell</t>
+        </is>
+      </c>
+      <c r="B88">
+        <f t="array" ref="B88:D88">INDEX([1]Uses!$A$1:$C$3,1,{1,2,3})</f>
+        <v>0</v>
+      </c>
+      <c r="C88">
+        <v>0</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>IDXliftSUM</t>
+        </is>
+      </c>
+      <c r="B89">
+        <f>SUM(INDEX([1]Uses!$A$1:$B$3,{1,2},1))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>IDXliftROWS</t>
+        </is>
+      </c>
+      <c r="B90">
+        <f>ROWS(INDEX([1]Uses!$A$1:$B$3,{1,2},1))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>IDXliftISREF</t>
+        </is>
+      </c>
+      <c r="B91">
+        <f>ISREF(INDEX([1]Uses!$A$1:$B$3,{1,2},1))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>IDXliftINDEX</t>
+        </is>
+      </c>
+      <c r="B92">
+        <f>INDEX(INDEX([1]Uses!$A$1:$B$3,{1,2},1),2)</f>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>